<commit_message>
Update blockchain and excel files
</commit_message>
<xml_diff>
--- a/backend/Blockchain/leader/alerts.xlsx
+++ b/backend/Blockchain/leader/alerts.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2598,6 +2598,82 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Keylogging</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>social enginnering</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>192.168.66.159</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2026-05-04T11:08:17</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Keylogging</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>social enginnering</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>192.168.66.159</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2026-05-04T11:08:17</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>